<commit_message>
Retrieval Rhythm: rättelser efter slutgranskning
Loggfältet rymmer ett helt läsår; frågorna gäller loggen men facit får
förklara; veckorna räknas på samma sätt i quiz, flerval och grid; KEY passar
öppna format; datum på LESSON-raden; loggmallen har ett tomt loggblad och
exemplet på eget blad, Notes märkt som ej för prompten; tillgänglighet i
formuläret; sidtestet bygger på en kopia; elevbladen märker lärarstegen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/downloads/retrieval-rhythm-log.xlsx
+++ b/assets/downloads/retrieval-rhythm-log.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,6 +427,408 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Key points</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Notes (not for the prompt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n"/>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n"/>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n"/>
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n"/>
+      <c r="B14" s="2" t="n"/>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n"/>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="n"/>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n"/>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n"/>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n"/>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n"/>
+      <c r="B29" s="2" t="n"/>
+      <c r="C29" s="2" t="n"/>
+      <c r="D29" s="2" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n"/>
+      <c r="B32" s="2" t="n"/>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n"/>
+      <c r="B33" s="2" t="n"/>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n"/>
+      <c r="B34" s="2" t="n"/>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n"/>
+      <c r="B35" s="2" t="n"/>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n"/>
+      <c r="B36" s="2" t="n"/>
+      <c r="C36" s="2" t="n"/>
+      <c r="D36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n"/>
+      <c r="B37" s="2" t="n"/>
+      <c r="C37" s="2" t="n"/>
+      <c r="D37" s="2" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n"/>
+      <c r="B38" s="2" t="n"/>
+      <c r="C38" s="2" t="n"/>
+      <c r="D38" s="2" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n"/>
+      <c r="B39" s="2" t="n"/>
+      <c r="C39" s="2" t="n"/>
+      <c r="D39" s="2" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n"/>
+      <c r="B40" s="2" t="n"/>
+      <c r="C40" s="2" t="n"/>
+      <c r="D40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n"/>
+      <c r="B41" s="2" t="n"/>
+      <c r="C41" s="2" t="n"/>
+      <c r="D41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n"/>
+      <c r="B42" s="2" t="n"/>
+      <c r="C42" s="2" t="n"/>
+      <c r="D42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n"/>
+      <c r="B44" s="2" t="n"/>
+      <c r="C44" s="2" t="n"/>
+      <c r="D44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n"/>
+      <c r="B45" s="2" t="n"/>
+      <c r="C45" s="2" t="n"/>
+      <c r="D45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n"/>
+      <c r="B46" s="2" t="n"/>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n"/>
+      <c r="B48" s="2" t="n"/>
+      <c r="C48" s="2" t="n"/>
+      <c r="D48" s="2" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n"/>
+      <c r="B49" s="2" t="n"/>
+      <c r="C49" s="2" t="n"/>
+      <c r="D49" s="2" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n"/>
+      <c r="B50" s="2" t="n"/>
+      <c r="C50" s="2" t="n"/>
+      <c r="D50" s="2" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n"/>
+      <c r="B51" s="2" t="n"/>
+      <c r="C51" s="2" t="n"/>
+      <c r="D51" s="2" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n"/>
+      <c r="B52" s="2" t="n"/>
+      <c r="C52" s="2" t="n"/>
+      <c r="D52" s="2" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="2" t="n"/>
+      <c r="D53" s="2" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="n"/>
+      <c r="D54" s="2" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n"/>
+      <c r="B55" s="2" t="n"/>
+      <c r="C55" s="2" t="n"/>
+      <c r="D55" s="2" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n"/>
+      <c r="B56" s="2" t="n"/>
+      <c r="C56" s="2" t="n"/>
+      <c r="D56" s="2" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n"/>
+      <c r="B57" s="2" t="n"/>
+      <c r="C57" s="2" t="n"/>
+      <c r="D57" s="2" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n"/>
+      <c r="B58" s="2" t="n"/>
+      <c r="C58" s="2" t="n"/>
+      <c r="D58" s="2" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
+      <c r="C59" s="2" t="n"/>
+      <c r="D59" s="2" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n"/>
+      <c r="B60" s="2" t="n"/>
+      <c r="C60" s="2" t="n"/>
+      <c r="D60" s="2" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n"/>
+      <c r="B61" s="2" t="n"/>
+      <c r="C61" s="2" t="n"/>
+      <c r="D61" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -453,7 +856,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Notes (not for the prompt)</t>
         </is>
       </c>
     </row>
@@ -966,7 +1369,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -988,14 +1391,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1. After each lesson, add a row: the date, the topic and two or three key points. Replace the example rows with your own.</t>
+          <t>1. After each lesson, add a row on the Log sheet: the date, the topic and two or three key points. The Example sheet shows what it can look like.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2. On Friday, copy the rows and paste them into the prompt builder at choosewise.education/retrieval-rhythm.</t>
+          <t>2. On Friday, copy columns A to C and paste them into the prompt builder at choosewise.education/retrieval-rhythm. Leave the Notes column out.</t>
         </is>
       </c>
     </row>

</xml_diff>